<commit_message>
Update JNJ data - 2026-09-06 16:10:47
</commit_message>
<xml_diff>
--- a/data/JNJ_data.xlsx
+++ b/data/JNJ_data.xlsx
@@ -4851,7 +4851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4972,25 +4972,45 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>book_value</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>price_to_book</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>earnings_growth</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>shares_outstanding</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -5050,7 +5070,7 @@
         <v>0.235</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.93</v>
+        <v>1.95</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -5074,29 +5094,41 @@
       <c r="W2" t="n">
         <v>1.089</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="n">
+        <v>35.284</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>7.80042</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2409898597</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Drug Manufacturers - General</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>https://www.jnj.com</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Johnson &amp; Johnson, together with its subsidiaries, engages in the research and development, manufacture, and sale of a range of products in the healthcare field worldwide. It operates in two segments, Innovative Medicine and MedTech. The Innovative Medicine segment offers products for various therapeutic areas, such as oncology, immunology, neuroscience, pulmonary hypertension, infectious diseases, and cardiovascular and metabolism distributed through retailers, wholesalers, distributors, hospitals, and healthcare professionals for prescription use. The MedTech segment provides a portfolio of products used in the surgery, orthopedic, cardiovascular, and vision fields distributed through wholesalers, hospitals and retailers, and used in the professional fields by physicians, nurses, hospitals, eye care professionals and clinics. This segment also offers products and enabling technologies that support joint reconstruction, trauma, spine, sports related injuries, and others, as well as open, laparoscopic, and robotic surgical procedures; instrumentation, energy devices, stapling systems, wound closure, biosurgery products, and digital and robotic technologies; breast aesthetics and reconstruction; contact lenses under the ACUVUE brand; intraocular lenses for cataract surgery, and other products used in cataract and refractive procedures under the TECNIS brand. The company was founded in 1886 and is based in New Brunswick, New Jersey.</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>2026-09-06 05:42:07</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:10:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update JNJ data - 2026-09-06 17:00:22
</commit_message>
<xml_diff>
--- a/data/JNJ_data.xlsx
+++ b/data/JNJ_data.xlsx
@@ -5072,15 +5072,11 @@
       <c r="Q2" t="n">
         <v>1.95</v>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="R2" t="n">
+        <v>0.21482</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.2919</v>
       </c>
       <c r="T2" t="n">
         <v>0.25742</v>
@@ -5128,7 +5124,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>2026-09-06 16:49:14</t>
+          <t>2026-09-06 16:59:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update JNJ data - 2026-09-06 22:21:27
</commit_message>
<xml_diff>
--- a/data/JNJ_data.xlsx
+++ b/data/JNJ_data.xlsx
@@ -4851,7 +4851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4992,25 +4992,40 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>enterprise_value</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -5102,29 +5117,38 @@
       <c r="AA2" t="n">
         <v>2409898597</v>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>97929003008</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>691554418688</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>34872000512</v>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Drug Manufacturers - General</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>https://www.jnj.com</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Johnson &amp; Johnson, together with its subsidiaries, engages in the research and development, manufacture, and sale of a range of products in the healthcare field worldwide. It operates in two segments, Innovative Medicine and MedTech. The Innovative Medicine segment offers products for various therapeutic areas, such as oncology, immunology, neuroscience, pulmonary hypertension, infectious diseases, and cardiovascular and metabolism distributed through retailers, wholesalers, distributors, hospitals, and healthcare professionals for prescription use. The MedTech segment provides a portfolio of products used in the surgery, orthopedic, cardiovascular, and vision fields distributed through wholesalers, hospitals and retailers, and used in the professional fields by physicians, nurses, hospitals, eye care professionals and clinics. This segment also offers products and enabling technologies that support joint reconstruction, trauma, spine, sports related injuries, and others, as well as open, laparoscopic, and robotic surgical procedures; instrumentation, energy devices, stapling systems, wound closure, biosurgery products, and digital and robotic technologies; breast aesthetics and reconstruction; contact lenses under the ACUVUE brand; intraocular lenses for cataract surgery, and other products used in cataract and refractive procedures under the TECNIS brand. The company was founded in 1886 and is based in New Brunswick, New Jersey.</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>2026-09-06 16:59:44</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>2026-09-06 22:20:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update JNJ data - 2026-09-08 08:53:13
</commit_message>
<xml_diff>
--- a/data/JNJ_data.xlsx
+++ b/data/JNJ_data.xlsx
@@ -472,16 +472,16 @@
         <v>45905</v>
       </c>
       <c r="B2" t="n">
-        <v>174.0770425638393</v>
+        <v>174.0770273418219</v>
       </c>
       <c r="C2" t="n">
-        <v>175.5537581707923</v>
+        <v>175.5537428196448</v>
       </c>
       <c r="D2" t="n">
-        <v>172.6687764611162</v>
+        <v>172.6687613622434</v>
       </c>
       <c r="E2" t="n">
-        <v>174.49755859375</v>
+        <v>174.4975433349609</v>
       </c>
       <c r="F2" t="n">
         <v>9733800</v>
@@ -498,16 +498,16 @@
         <v>45908</v>
       </c>
       <c r="B3" t="n">
-        <v>173.4511589867753</v>
+        <v>173.4511437939455</v>
       </c>
       <c r="C3" t="n">
-        <v>175.4950938415212</v>
+        <v>175.4950784696603</v>
       </c>
       <c r="D3" t="n">
-        <v>172.8057011623818</v>
+        <v>172.8056860260886</v>
       </c>
       <c r="E3" t="n">
-        <v>174.2041931152344</v>
+        <v>174.2041778564453</v>
       </c>
       <c r="F3" t="n">
         <v>8382500</v>
@@ -524,16 +524,16 @@
         <v>45909</v>
       </c>
       <c r="B4" t="n">
-        <v>174.0770398088306</v>
+        <v>174.0770551572955</v>
       </c>
       <c r="C4" t="n">
-        <v>174.165052708233</v>
+        <v>174.1650680644581</v>
       </c>
       <c r="D4" t="n">
-        <v>172.561197432737</v>
+        <v>172.5612126475493</v>
       </c>
       <c r="E4" t="n">
-        <v>173.0599670410156</v>
+        <v>173.0599822998047</v>
       </c>
       <c r="F4" t="n">
         <v>6005700</v>
@@ -576,16 +576,16 @@
         <v>45911</v>
       </c>
       <c r="B6" t="n">
-        <v>171.8766472653515</v>
+        <v>171.8766172179321</v>
       </c>
       <c r="C6" t="n">
-        <v>174.9083323610806</v>
+        <v>174.908301783663</v>
       </c>
       <c r="D6" t="n">
-        <v>171.759296719517</v>
+        <v>171.7592666926129</v>
       </c>
       <c r="E6" t="n">
-        <v>174.5660400390625</v>
+        <v>174.5660095214844</v>
       </c>
       <c r="F6" t="n">
         <v>5792500</v>
@@ -602,16 +602,16 @@
         <v>45912</v>
       </c>
       <c r="B7" t="n">
-        <v>173.7934495446803</v>
+        <v>173.7934343158836</v>
       </c>
       <c r="C7" t="n">
-        <v>174.8594234144472</v>
+        <v>174.8594080922437</v>
       </c>
       <c r="D7" t="n">
-        <v>172.8252628178507</v>
+        <v>172.8252476738922</v>
       </c>
       <c r="E7" t="n">
-        <v>174.1357269287109</v>
+        <v>174.1357116699219</v>
       </c>
       <c r="F7" t="n">
         <v>7220200</v>
@@ -628,16 +628,16 @@
         <v>45915</v>
       </c>
       <c r="B8" t="n">
-        <v>173.8423161383384</v>
+        <v>173.8423314280924</v>
       </c>
       <c r="C8" t="n">
-        <v>175.0452187336727</v>
+        <v>175.0452341292242</v>
       </c>
       <c r="D8" t="n">
-        <v>173.0306068383358</v>
+        <v>173.0306220566984</v>
       </c>
       <c r="E8" t="n">
-        <v>173.4902496337891</v>
+        <v>173.4902648925781</v>
       </c>
       <c r="F8" t="n">
         <v>4768100</v>
@@ -706,16 +706,16 @@
         <v>45918</v>
       </c>
       <c r="B11" t="n">
-        <v>172.7078974682877</v>
+        <v>172.7079129408542</v>
       </c>
       <c r="C11" t="n">
-        <v>173.1186392474049</v>
+        <v>173.118654756769</v>
       </c>
       <c r="D11" t="n">
-        <v>170.0380535202773</v>
+        <v>170.0380687536577</v>
       </c>
       <c r="E11" t="n">
-        <v>170.3216705322266</v>
+        <v>170.3216857910156</v>
       </c>
       <c r="F11" t="n">
         <v>8200900</v>
@@ -784,16 +784,16 @@
         <v>45923</v>
       </c>
       <c r="B14" t="n">
-        <v>171.0355980210813</v>
+        <v>171.0355829083302</v>
       </c>
       <c r="C14" t="n">
-        <v>173.0697586837889</v>
+        <v>173.0697433912989</v>
       </c>
       <c r="D14" t="n">
-        <v>170.9769227489119</v>
+        <v>170.9769076413454</v>
       </c>
       <c r="E14" t="n">
-        <v>172.6883544921875</v>
+        <v>172.6883392333984</v>
       </c>
       <c r="F14" t="n">
         <v>8350400</v>
@@ -810,16 +810,16 @@
         <v>45924</v>
       </c>
       <c r="B15" t="n">
-        <v>172.2580322171388</v>
+        <v>172.2580474284301</v>
       </c>
       <c r="C15" t="n">
-        <v>173.0501781580241</v>
+        <v>173.0501934392661</v>
       </c>
       <c r="D15" t="n">
-        <v>171.8668538263927</v>
+        <v>171.8668690031409</v>
       </c>
       <c r="E15" t="n">
-        <v>172.7959136962891</v>
+        <v>172.7959289550781</v>
       </c>
       <c r="F15" t="n">
         <v>6676800</v>
@@ -1018,16 +1018,16 @@
         <v>45936</v>
       </c>
       <c r="B23" t="n">
-        <v>183.8566604823808</v>
+        <v>183.8566452365672</v>
       </c>
       <c r="C23" t="n">
-        <v>185.7343437349051</v>
+        <v>185.7343283333897</v>
       </c>
       <c r="D23" t="n">
-        <v>183.2405403023728</v>
+        <v>183.2405251076493</v>
       </c>
       <c r="E23" t="n">
-        <v>184.0131378173828</v>
+        <v>184.0131225585938</v>
       </c>
       <c r="F23" t="n">
         <v>5806100</v>
@@ -1044,16 +1044,16 @@
         <v>45937</v>
       </c>
       <c r="B24" t="n">
-        <v>179.7198952882722</v>
+        <v>179.7198804430833</v>
       </c>
       <c r="C24" t="n">
-        <v>185.0595539364086</v>
+        <v>185.0595386501542</v>
       </c>
       <c r="D24" t="n">
-        <v>178.908185875973</v>
+        <v>178.9081710978327</v>
       </c>
       <c r="E24" t="n">
-        <v>184.72705078125</v>
+        <v>184.7270355224609</v>
       </c>
       <c r="F24" t="n">
         <v>8776800</v>
@@ -1070,16 +1070,16 @@
         <v>45938</v>
       </c>
       <c r="B25" t="n">
-        <v>184.7074643396089</v>
+        <v>184.707479532436</v>
       </c>
       <c r="C25" t="n">
-        <v>186.0277174802343</v>
+        <v>186.0277327816568</v>
       </c>
       <c r="D25" t="n">
-        <v>184.1206967723854</v>
+        <v>184.1207119169489</v>
       </c>
       <c r="E25" t="n">
-        <v>185.5093994140625</v>
+        <v>185.5094146728516</v>
       </c>
       <c r="F25" t="n">
         <v>5751200</v>
@@ -1148,16 +1148,16 @@
         <v>45943</v>
       </c>
       <c r="B28" t="n">
-        <v>185.646323339356</v>
+        <v>185.6463081660922</v>
       </c>
       <c r="C28" t="n">
-        <v>187.0839270863694</v>
+        <v>187.0839117956073</v>
       </c>
       <c r="D28" t="n">
-        <v>185.1084418485517</v>
+        <v>185.1084267192501</v>
       </c>
       <c r="E28" t="n">
-        <v>186.6927337646484</v>
+        <v>186.6927185058594</v>
       </c>
       <c r="F28" t="n">
         <v>7979500</v>
@@ -1226,16 +1226,16 @@
         <v>45946</v>
       </c>
       <c r="B31" t="n">
-        <v>187.1230558646578</v>
+        <v>187.1230406678187</v>
       </c>
       <c r="C31" t="n">
-        <v>188.7953757558051</v>
+        <v>188.7953604231518</v>
       </c>
       <c r="D31" t="n">
-        <v>186.2331077651437</v>
+        <v>186.2330926405801</v>
       </c>
       <c r="E31" t="n">
-        <v>187.8858642578125</v>
+        <v>187.8858489990234</v>
       </c>
       <c r="F31" t="n">
         <v>10611800</v>
@@ -1278,16 +1278,16 @@
         <v>45950</v>
       </c>
       <c r="B33" t="n">
-        <v>189.2354242017374</v>
+        <v>189.2354394431975</v>
       </c>
       <c r="C33" t="n">
-        <v>190.1938216550539</v>
+        <v>190.1938369737056</v>
       </c>
       <c r="D33" t="n">
-        <v>188.0912117995895</v>
+        <v>188.0912269488921</v>
       </c>
       <c r="E33" t="n">
-        <v>189.4505767822266</v>
+        <v>189.4505920410156</v>
       </c>
       <c r="F33" t="n">
         <v>8034700</v>
@@ -1304,16 +1304,16 @@
         <v>45951</v>
       </c>
       <c r="B34" t="n">
-        <v>188.756223952035</v>
+        <v>188.7562393006838</v>
       </c>
       <c r="C34" t="n">
-        <v>189.2843311834856</v>
+        <v>189.2843465750772</v>
       </c>
       <c r="D34" t="n">
-        <v>187.5435620120352</v>
+        <v>187.5435772620767</v>
       </c>
       <c r="E34" t="n">
-        <v>187.6511383056641</v>
+        <v>187.6511535644531</v>
       </c>
       <c r="F34" t="n">
         <v>6716000</v>
@@ -1330,16 +1330,16 @@
         <v>45952</v>
       </c>
       <c r="B35" t="n">
-        <v>187.768489042997</v>
+        <v>187.7685194118937</v>
       </c>
       <c r="C35" t="n">
-        <v>189.186529335124</v>
+        <v>189.1865599333687</v>
       </c>
       <c r="D35" t="n">
-        <v>187.553336455502</v>
+        <v>187.5533667896008</v>
       </c>
       <c r="E35" t="n">
-        <v>188.6877746582031</v>
+        <v>188.6878051757812</v>
       </c>
       <c r="F35" t="n">
         <v>6343100</v>
@@ -1356,16 +1356,16 @@
         <v>45953</v>
       </c>
       <c r="B36" t="n">
-        <v>188.3161623201141</v>
+        <v>188.3161470541903</v>
       </c>
       <c r="C36" t="n">
-        <v>189.7244285069409</v>
+        <v>189.7244131268554</v>
       </c>
       <c r="D36" t="n">
-        <v>187.3186379506951</v>
+        <v>187.318622765636</v>
       </c>
       <c r="E36" t="n">
-        <v>188.2281494140625</v>
+        <v>188.2281341552734</v>
       </c>
       <c r="F36" t="n">
         <v>8882500</v>
@@ -1382,16 +1382,16 @@
         <v>45954</v>
       </c>
       <c r="B37" t="n">
-        <v>187.9640832263789</v>
+        <v>187.9640678233363</v>
       </c>
       <c r="C37" t="n">
-        <v>188.0716595229833</v>
+        <v>188.0716441111252</v>
       </c>
       <c r="D37" t="n">
-        <v>185.2453531003753</v>
+        <v>185.2453379201237</v>
       </c>
       <c r="E37" t="n">
-        <v>186.2037506103516</v>
+        <v>186.2037353515625</v>
       </c>
       <c r="F37" t="n">
         <v>6903400</v>
@@ -1460,16 +1460,16 @@
         <v>45959</v>
       </c>
       <c r="B40" t="n">
-        <v>182.5852901845839</v>
+        <v>182.5853054515495</v>
       </c>
       <c r="C40" t="n">
-        <v>182.9764834833836</v>
+        <v>182.9764987830591</v>
       </c>
       <c r="D40" t="n">
-        <v>180.5902565894498</v>
+        <v>180.5902716895996</v>
       </c>
       <c r="E40" t="n">
-        <v>182.4875030517578</v>
+        <v>182.4875183105469</v>
       </c>
       <c r="F40" t="n">
         <v>10551100</v>
@@ -1486,16 +1486,16 @@
         <v>45960</v>
       </c>
       <c r="B41" t="n">
-        <v>182.9569302033718</v>
+        <v>182.9569151035874</v>
       </c>
       <c r="C41" t="n">
-        <v>185.2062432977132</v>
+        <v>185.2062280122887</v>
       </c>
       <c r="D41" t="n">
-        <v>182.7906786381269</v>
+        <v>182.7906635520636</v>
       </c>
       <c r="E41" t="n">
-        <v>184.8835144042969</v>
+        <v>184.8834991455078</v>
       </c>
       <c r="F41" t="n">
         <v>7072500</v>
@@ -1538,16 +1538,16 @@
         <v>45964</v>
       </c>
       <c r="B43" t="n">
-        <v>184.8346326024117</v>
+        <v>184.834617119156</v>
       </c>
       <c r="C43" t="n">
-        <v>184.8639702391834</v>
+        <v>184.8639547534701</v>
       </c>
       <c r="D43" t="n">
-        <v>181.4313324343818</v>
+        <v>181.4313172362143</v>
       </c>
       <c r="E43" t="n">
-        <v>182.1550140380859</v>
+        <v>182.1549987792969</v>
       </c>
       <c r="F43" t="n">
         <v>7542600</v>
@@ -1668,16 +1668,16 @@
         <v>45971</v>
       </c>
       <c r="B48" t="n">
-        <v>181.9007248187872</v>
+        <v>181.9007398823969</v>
       </c>
       <c r="C48" t="n">
-        <v>184.2673883725038</v>
+        <v>184.2674036321023</v>
       </c>
       <c r="D48" t="n">
-        <v>181.0401144637998</v>
+        <v>181.0401294561404</v>
       </c>
       <c r="E48" t="n">
-        <v>184.2576141357422</v>
+        <v>184.2576293945312</v>
       </c>
       <c r="F48" t="n">
         <v>5323800</v>
@@ -1720,16 +1720,16 @@
         <v>45973</v>
       </c>
       <c r="B50" t="n">
-        <v>189.0985363418636</v>
+        <v>189.0985059859865</v>
       </c>
       <c r="C50" t="n">
-        <v>191.24027328305</v>
+        <v>191.2402425833612</v>
       </c>
       <c r="D50" t="n">
-        <v>188.8149342225856</v>
+        <v>188.814903912235</v>
       </c>
       <c r="E50" t="n">
-        <v>190.1058349609375</v>
+        <v>190.1058044433594</v>
       </c>
       <c r="F50" t="n">
         <v>8803000</v>
@@ -1772,16 +1772,16 @@
         <v>45975</v>
       </c>
       <c r="B52" t="n">
-        <v>190.7023657548931</v>
+        <v>190.7023809412554</v>
       </c>
       <c r="C52" t="n">
-        <v>192.8343132451486</v>
+        <v>192.8343286012861</v>
       </c>
       <c r="D52" t="n">
-        <v>189.2843255068563</v>
+        <v>189.2843405802947</v>
       </c>
       <c r="E52" t="n">
-        <v>191.6118621826172</v>
+        <v>191.6118774414062</v>
       </c>
       <c r="F52" t="n">
         <v>8824800</v>
@@ -1902,16 +1902,16 @@
         <v>45982</v>
       </c>
       <c r="B57" t="n">
-        <v>199.4649249339953</v>
+        <v>199.4649096707152</v>
       </c>
       <c r="C57" t="n">
-        <v>202.3792444306165</v>
+        <v>202.3792289443294</v>
       </c>
       <c r="D57" t="n">
-        <v>198.5163016043988</v>
+        <v>198.5162864137085</v>
       </c>
       <c r="E57" t="n">
-        <v>199.4062347412109</v>
+        <v>199.4062194824219</v>
       </c>
       <c r="F57" t="n">
         <v>13189100</v>
@@ -1928,16 +1928,16 @@
         <v>45985</v>
       </c>
       <c r="B58" t="n">
-        <v>199.2204251313988</v>
+        <v>199.2204100458954</v>
       </c>
       <c r="C58" t="n">
-        <v>201.5772996022027</v>
+        <v>201.5772843382305</v>
       </c>
       <c r="D58" t="n">
-        <v>198.5260663138595</v>
+        <v>198.5260512809348</v>
       </c>
       <c r="E58" t="n">
-        <v>201.5088500976562</v>
+        <v>201.5088348388672</v>
       </c>
       <c r="F58" t="n">
         <v>14803900</v>
@@ -1954,16 +1954,16 @@
         <v>45986</v>
       </c>
       <c r="B59" t="n">
-        <v>201.9320337594338</v>
+        <v>201.9320489082132</v>
       </c>
       <c r="C59" t="n">
-        <v>204.4318344688182</v>
+        <v>204.4318498051307</v>
       </c>
       <c r="D59" t="n">
-        <v>201.9320337594338</v>
+        <v>201.9320489082132</v>
       </c>
       <c r="E59" t="n">
-        <v>203.3984527587891</v>
+        <v>203.3984680175781</v>
       </c>
       <c r="F59" t="n">
         <v>10275300</v>
@@ -2110,16 +2110,16 @@
         <v>45995</v>
       </c>
       <c r="B65" t="n">
-        <v>201.3513800209524</v>
+        <v>201.35139543875</v>
       </c>
       <c r="C65" t="n">
-        <v>201.6171101829578</v>
+        <v>201.6171256211029</v>
       </c>
       <c r="D65" t="n">
-        <v>198.516980022795</v>
+        <v>198.5169952235581</v>
       </c>
       <c r="E65" t="n">
-        <v>199.2747802734375</v>
+        <v>199.2747955322266</v>
       </c>
       <c r="F65" t="n">
         <v>9049900</v>
@@ -2292,16 +2292,16 @@
         <v>46006</v>
       </c>
       <c r="B72" t="n">
-        <v>207.0202168563343</v>
+        <v>207.020201869705</v>
       </c>
       <c r="C72" t="n">
-        <v>211.7835972337083</v>
+        <v>211.7835819022478</v>
       </c>
       <c r="D72" t="n">
-        <v>205.7014173161141</v>
+        <v>205.7014024249555</v>
       </c>
       <c r="E72" t="n">
-        <v>210.7797393798828</v>
+        <v>210.7797241210938</v>
       </c>
       <c r="F72" t="n">
         <v>8467000</v>
@@ -2344,16 +2344,16 @@
         <v>46008</v>
       </c>
       <c r="B74" t="n">
-        <v>206.0753964132944</v>
+        <v>206.0753812226996</v>
       </c>
       <c r="C74" t="n">
-        <v>208.1716837329721</v>
+        <v>208.171668387852</v>
       </c>
       <c r="D74" t="n">
-        <v>205.1601253407421</v>
+        <v>205.1601102176154</v>
       </c>
       <c r="E74" t="n">
-        <v>207.0005187988281</v>
+        <v>207.0005035400391</v>
       </c>
       <c r="F74" t="n">
         <v>8457600</v>
@@ -2370,16 +2370,16 @@
         <v>46009</v>
       </c>
       <c r="B75" t="n">
-        <v>206.478915988136</v>
+        <v>206.4789006202035</v>
       </c>
       <c r="C75" t="n">
-        <v>207.7189650641044</v>
+        <v>207.7189496038768</v>
       </c>
       <c r="D75" t="n">
-        <v>204.4712003216206</v>
+        <v>204.4711851031195</v>
       </c>
       <c r="E75" t="n">
-        <v>205.0124969482422</v>
+        <v>205.0124816894531</v>
       </c>
       <c r="F75" t="n">
         <v>7499900</v>
@@ -2422,16 +2422,16 @@
         <v>46013</v>
       </c>
       <c r="B77" t="n">
-        <v>202.8670125241163</v>
+        <v>202.8669973529117</v>
       </c>
       <c r="C77" t="n">
-        <v>204.7861414522214</v>
+        <v>204.7861261374966</v>
       </c>
       <c r="D77" t="n">
-        <v>202.2469804791725</v>
+        <v>202.2469653543363</v>
       </c>
       <c r="E77" t="n">
-        <v>204.0381774902344</v>
+        <v>204.0381622314453</v>
       </c>
       <c r="F77" t="n">
         <v>8187800</v>
@@ -2448,16 +2448,16 @@
         <v>46014</v>
       </c>
       <c r="B78" t="n">
-        <v>201.7745733053134</v>
+        <v>201.7745885077481</v>
       </c>
       <c r="C78" t="n">
-        <v>203.2606648620441</v>
+        <v>203.2606801764464</v>
       </c>
       <c r="D78" t="n">
-        <v>200.062111796116</v>
+        <v>200.0621268695276</v>
       </c>
       <c r="E78" t="n">
-        <v>202.5225372314453</v>
+        <v>202.5225524902344</v>
       </c>
       <c r="F78" t="n">
         <v>7047300</v>
@@ -2474,16 +2474,16 @@
         <v>46015</v>
       </c>
       <c r="B79" t="n">
-        <v>202.739053555574</v>
+        <v>202.7390686836449</v>
       </c>
       <c r="C79" t="n">
-        <v>204.648346074342</v>
+        <v>204.6483613448813</v>
       </c>
       <c r="D79" t="n">
-        <v>202.3158675938084</v>
+        <v>202.3158826903017</v>
       </c>
       <c r="E79" t="n">
-        <v>204.4908752441406</v>
+        <v>204.4908905029297</v>
       </c>
       <c r="F79" t="n">
         <v>2376500</v>
@@ -2552,16 +2552,16 @@
         <v>46021</v>
       </c>
       <c r="B82" t="n">
-        <v>204.2251519205988</v>
+        <v>204.2251366175628</v>
       </c>
       <c r="C82" t="n">
-        <v>204.4023103648072</v>
+        <v>204.4022950484963</v>
       </c>
       <c r="D82" t="n">
-        <v>203.2508330378112</v>
+        <v>203.2508178077831</v>
       </c>
       <c r="E82" t="n">
-        <v>203.6346588134766</v>
+        <v>203.6346435546875</v>
       </c>
       <c r="F82" t="n">
         <v>3937400</v>
@@ -2578,16 +2578,16 @@
         <v>46022</v>
       </c>
       <c r="B83" t="n">
-        <v>203.6346510317296</v>
+        <v>203.6346662875698</v>
       </c>
       <c r="C83" t="n">
-        <v>204.2153078209129</v>
+        <v>204.2153231202547</v>
       </c>
       <c r="D83" t="n">
-        <v>203.103190736659</v>
+        <v>203.1032059526835</v>
       </c>
       <c r="E83" t="n">
-        <v>203.6740112304688</v>
+        <v>203.6740264892578</v>
       </c>
       <c r="F83" t="n">
         <v>4083800</v>
@@ -2604,16 +2604,16 @@
         <v>46024</v>
       </c>
       <c r="B84" t="n">
-        <v>203.546094226423</v>
+        <v>203.5460790066363</v>
       </c>
       <c r="C84" t="n">
-        <v>204.1070634486917</v>
+        <v>204.1070481869595</v>
       </c>
       <c r="D84" t="n">
-        <v>200.4557852869147</v>
+        <v>200.4557702982002</v>
       </c>
       <c r="E84" t="n">
-        <v>204.0677032470703</v>
+        <v>204.0676879882812</v>
       </c>
       <c r="F84" t="n">
         <v>6325500</v>
@@ -2656,16 +2656,16 @@
         <v>46028</v>
       </c>
       <c r="B86" t="n">
-        <v>201.3612227968269</v>
+        <v>201.3612380414601</v>
       </c>
       <c r="C86" t="n">
-        <v>203.4378224562984</v>
+        <v>203.4378378581467</v>
       </c>
       <c r="D86" t="n">
-        <v>200.8888103027919</v>
+        <v>200.8888255116597</v>
       </c>
       <c r="E86" t="n">
-        <v>201.5482025146484</v>
+        <v>201.5482177734375</v>
       </c>
       <c r="F86" t="n">
         <v>8107900</v>
@@ -2734,16 +2734,16 @@
         <v>46031</v>
       </c>
       <c r="B89" t="n">
-        <v>202.6504838830927</v>
+        <v>202.6504992553581</v>
       </c>
       <c r="C89" t="n">
-        <v>203.4279717120081</v>
+        <v>203.4279871432506</v>
       </c>
       <c r="D89" t="n">
-        <v>200.7805515444468</v>
+        <v>200.7805667748665</v>
       </c>
       <c r="E89" t="n">
-        <v>201.154541015625</v>
+        <v>201.1545562744141</v>
       </c>
       <c r="F89" t="n">
         <v>6154300</v>
@@ -2760,16 +2760,16 @@
         <v>46034</v>
       </c>
       <c r="B90" t="n">
-        <v>202.2961890410606</v>
+        <v>202.2962039964493</v>
       </c>
       <c r="C90" t="n">
-        <v>206.5773204309254</v>
+        <v>206.5773357028104</v>
       </c>
       <c r="D90" t="n">
-        <v>200.6231026927027</v>
+        <v>200.6231175244031</v>
       </c>
       <c r="E90" t="n">
-        <v>206.4001770019531</v>
+        <v>206.4001922607422</v>
       </c>
       <c r="F90" t="n">
         <v>11794300</v>
@@ -2916,16 +2916,16 @@
         <v>46043</v>
       </c>
       <c r="B96" t="n">
-        <v>207.6599020836601</v>
+        <v>207.659916851811</v>
       </c>
       <c r="C96" t="n">
-        <v>215.218321643167</v>
+        <v>215.2183369488501</v>
       </c>
       <c r="D96" t="n">
-        <v>207.1678170076325</v>
+        <v>207.1678317407877</v>
       </c>
       <c r="E96" t="n">
-        <v>214.5589294433594</v>
+        <v>214.5589447021484</v>
       </c>
       <c r="F96" t="n">
         <v>14762900</v>
@@ -2942,16 +2942,16 @@
         <v>46044</v>
       </c>
       <c r="B97" t="n">
-        <v>215.3069079934484</v>
+        <v>215.3069232717918</v>
       </c>
       <c r="C97" t="n">
-        <v>218.6530804976869</v>
+        <v>218.6530960134773</v>
       </c>
       <c r="D97" t="n">
-        <v>214.6475157947938</v>
+        <v>214.6475310263463</v>
       </c>
       <c r="E97" t="n">
-        <v>215.0313415527344</v>
+        <v>215.0313568115234</v>
       </c>
       <c r="F97" t="n">
         <v>13160000</v>
@@ -2994,16 +2994,16 @@
         <v>46048</v>
       </c>
       <c r="B99" t="n">
-        <v>216.7241347564745</v>
+        <v>216.7241195858665</v>
       </c>
       <c r="C99" t="n">
-        <v>218.5153167809881</v>
+        <v>218.515301484998</v>
       </c>
       <c r="D99" t="n">
-        <v>216.5174523988691</v>
+        <v>216.5174372427288</v>
       </c>
       <c r="E99" t="n">
-        <v>217.9838714599609</v>
+        <v>217.9838562011719</v>
       </c>
       <c r="F99" t="n">
         <v>6856700</v>
@@ -3098,16 +3098,16 @@
         <v>46052</v>
       </c>
       <c r="B103" t="n">
-        <v>224.6466859457881</v>
+        <v>224.6466706191826</v>
       </c>
       <c r="C103" t="n">
-        <v>224.8828922015737</v>
+        <v>224.8828768588529</v>
       </c>
       <c r="D103" t="n">
-        <v>221.7630744488117</v>
+        <v>221.7630593189417</v>
       </c>
       <c r="E103" t="n">
-        <v>223.6526794433594</v>
+        <v>223.6526641845703</v>
       </c>
       <c r="F103" t="n">
         <v>11045500</v>
@@ -3124,16 +3124,16 @@
         <v>46055</v>
       </c>
       <c r="B104" t="n">
-        <v>224.7057483906486</v>
+        <v>224.7057634887497</v>
       </c>
       <c r="C104" t="n">
-        <v>227.530312073188</v>
+        <v>227.530327361073</v>
       </c>
       <c r="D104" t="n">
-        <v>223.6526790631295</v>
+        <v>223.6526940904743</v>
       </c>
       <c r="E104" t="n">
-        <v>227.0972747802734</v>
+        <v>227.0972900390625</v>
       </c>
       <c r="F104" t="n">
         <v>8187500</v>
@@ -3176,16 +3176,16 @@
         <v>46057</v>
       </c>
       <c r="B106" t="n">
-        <v>231.2800013484118</v>
+        <v>231.2799860551316</v>
       </c>
       <c r="C106" t="n">
-        <v>232.0968644318395</v>
+        <v>232.0968490845446</v>
       </c>
       <c r="D106" t="n">
-        <v>229.2526131010531</v>
+        <v>229.252597941833</v>
       </c>
       <c r="E106" t="n">
-        <v>230.7583923339844</v>
+        <v>230.7583770751953</v>
       </c>
       <c r="F106" t="n">
         <v>8641400</v>
@@ -3254,16 +3254,16 @@
         <v>46062</v>
       </c>
       <c r="B109" t="n">
-        <v>236.4468956382332</v>
+        <v>236.4468802764997</v>
       </c>
       <c r="C109" t="n">
-        <v>236.9291444528193</v>
+        <v>236.9291290597546</v>
       </c>
       <c r="D109" t="n">
-        <v>233.2877026206608</v>
+        <v>233.2876874641771</v>
       </c>
       <c r="E109" t="n">
-        <v>234.8623809814453</v>
+        <v>234.8623657226562</v>
       </c>
       <c r="F109" t="n">
         <v>9378500</v>
@@ -3332,16 +3332,16 @@
         <v>46065</v>
       </c>
       <c r="B112" t="n">
-        <v>236.6732529591429</v>
+        <v>236.6732379543034</v>
       </c>
       <c r="C112" t="n">
-        <v>242.4503424271597</v>
+        <v>242.4503270560588</v>
       </c>
       <c r="D112" t="n">
-        <v>235.8859137708501</v>
+        <v>235.8858988159272</v>
       </c>
       <c r="E112" t="n">
-        <v>240.6788330078125</v>
+        <v>240.6788177490234</v>
       </c>
       <c r="F112" t="n">
         <v>10254300</v>
@@ -3358,16 +3358,16 @@
         <v>46066</v>
       </c>
       <c r="B113" t="n">
-        <v>240.7181753030812</v>
+        <v>240.7181906333224</v>
       </c>
       <c r="C113" t="n">
-        <v>241.0724771605951</v>
+        <v>241.0724925134001</v>
       </c>
       <c r="D113" t="n">
-        <v>238.7695225953774</v>
+        <v>238.7695378015177</v>
       </c>
       <c r="E113" t="n">
-        <v>239.5962219238281</v>
+        <v>239.5962371826172</v>
       </c>
       <c r="F113" t="n">
         <v>13268500</v>
@@ -3488,16 +3488,16 @@
         <v>46076</v>
       </c>
       <c r="B118" t="n">
-        <v>239.7733870753068</v>
+        <v>239.7734021969262</v>
       </c>
       <c r="C118" t="n">
-        <v>242.9030410566114</v>
+        <v>242.9030563756065</v>
       </c>
       <c r="D118" t="n">
-        <v>238.7596929857211</v>
+        <v>238.7597080434106</v>
       </c>
       <c r="E118" t="n">
-        <v>241.9483947753906</v>
+        <v>241.9484100341797</v>
       </c>
       <c r="F118" t="n">
         <v>9622700</v>
@@ -3514,16 +3514,16 @@
         <v>46077</v>
       </c>
       <c r="B119" t="n">
-        <v>242.7498156695138</v>
+        <v>242.7498308706833</v>
       </c>
       <c r="C119" t="n">
-        <v>244.6296736547229</v>
+        <v>244.6296889736104</v>
       </c>
       <c r="D119" t="n">
-        <v>241.9483872724562</v>
+        <v>241.9484024234396</v>
       </c>
       <c r="E119" t="n">
-        <v>243.6699523925781</v>
+        <v>243.6699676513672</v>
       </c>
       <c r="F119" t="n">
         <v>7246300</v>
@@ -3540,16 +3540,16 @@
         <v>46078</v>
       </c>
       <c r="B120" t="n">
-        <v>242.2650040664713</v>
+        <v>242.2650193059668</v>
       </c>
       <c r="C120" t="n">
-        <v>244.629674532896</v>
+        <v>244.6296899211394</v>
       </c>
       <c r="D120" t="n">
-        <v>241.1370862518812</v>
+        <v>241.1371014204259</v>
       </c>
       <c r="E120" t="n">
-        <v>242.5717163085938</v>
+        <v>242.5717315673828</v>
       </c>
       <c r="F120" t="n">
         <v>7698200</v>
@@ -3566,16 +3566,16 @@
         <v>46079</v>
       </c>
       <c r="B121" t="n">
-        <v>242.5123588943122</v>
+        <v>242.5123742558835</v>
       </c>
       <c r="C121" t="n">
-        <v>242.8685442682355</v>
+        <v>242.8685596523689</v>
       </c>
       <c r="D121" t="n">
-        <v>239.4551099080992</v>
+        <v>239.4551250760139</v>
       </c>
       <c r="E121" t="n">
-        <v>240.8897399902344</v>
+        <v>240.8897552490234</v>
       </c>
       <c r="F121" t="n">
         <v>7172600</v>
@@ -3670,16 +3670,16 @@
         <v>46085</v>
       </c>
       <c r="B125" t="n">
-        <v>243.145575843863</v>
+        <v>243.1455911306439</v>
       </c>
       <c r="C125" t="n">
-        <v>243.9568928450567</v>
+        <v>243.9569081828458</v>
       </c>
       <c r="D125" t="n">
-        <v>240.6028050981046</v>
+        <v>240.6028202250193</v>
       </c>
       <c r="E125" t="n">
-        <v>242.7003479003906</v>
+        <v>242.7003631591797</v>
       </c>
       <c r="F125" t="n">
         <v>5768000</v>
@@ -3696,16 +3696,16 @@
         <v>46086</v>
       </c>
       <c r="B126" t="n">
-        <v>240.0586452528019</v>
+        <v>240.0586607026203</v>
       </c>
       <c r="C126" t="n">
-        <v>240.424719212307</v>
+        <v>240.4247346856854</v>
       </c>
       <c r="D126" t="n">
-        <v>233.4296388594088</v>
+        <v>233.4296538825942</v>
       </c>
       <c r="E126" t="n">
-        <v>237.0904388427734</v>
+        <v>237.0904541015625</v>
       </c>
       <c r="F126" t="n">
         <v>9375400</v>
@@ -3722,16 +3722,16 @@
         <v>46087</v>
       </c>
       <c r="B127" t="n">
-        <v>235.596428770922</v>
+        <v>235.5964438849938</v>
       </c>
       <c r="C127" t="n">
-        <v>238.2381306285037</v>
+        <v>238.238145912047</v>
       </c>
       <c r="D127" t="n">
-        <v>232.9349346436922</v>
+        <v>232.9349495870229</v>
       </c>
       <c r="E127" t="n">
-        <v>237.8522644042969</v>
+        <v>237.8522796630859</v>
       </c>
       <c r="F127" t="n">
         <v>7179800</v>
@@ -3748,16 +3748,16 @@
         <v>46090</v>
       </c>
       <c r="B128" t="n">
-        <v>238.3173005129137</v>
+        <v>238.3172853623119</v>
       </c>
       <c r="C128" t="n">
-        <v>241.5031767703235</v>
+        <v>241.5031614171852</v>
       </c>
       <c r="D128" t="n">
-        <v>237.4960948841201</v>
+        <v>237.496079785725</v>
       </c>
       <c r="E128" t="n">
-        <v>240.0190734863281</v>
+        <v>240.0190582275391</v>
       </c>
       <c r="F128" t="n">
         <v>7844000</v>
@@ -3826,16 +3826,16 @@
         <v>46093</v>
       </c>
       <c r="B131" t="n">
-        <v>238.9010593075404</v>
+        <v>238.9010440853151</v>
       </c>
       <c r="C131" t="n">
-        <v>241.8098890629796</v>
+        <v>241.8098736554103</v>
       </c>
       <c r="D131" t="n">
-        <v>237.7533491444783</v>
+        <v>237.7533339953824</v>
       </c>
       <c r="E131" t="n">
-        <v>239.4748992919922</v>
+        <v>239.4748840332031</v>
       </c>
       <c r="F131" t="n">
         <v>7710200</v>
@@ -3852,16 +3852,16 @@
         <v>46094</v>
       </c>
       <c r="B132" t="n">
-        <v>241.6219129804633</v>
+        <v>241.6218975517249</v>
       </c>
       <c r="C132" t="n">
-        <v>242.9872777226232</v>
+        <v>242.9872622066995</v>
       </c>
       <c r="D132" t="n">
-        <v>238.940626430393</v>
+        <v>238.9406111728678</v>
       </c>
       <c r="E132" t="n">
-        <v>238.9604187011719</v>
+        <v>238.9604034423828</v>
       </c>
       <c r="F132" t="n">
         <v>6415300</v>
@@ -3878,16 +3878,16 @@
         <v>46097</v>
       </c>
       <c r="B133" t="n">
-        <v>241.3349760333344</v>
+        <v>241.3349607287423</v>
       </c>
       <c r="C133" t="n">
-        <v>242.4628939057684</v>
+        <v>242.4628785296478</v>
       </c>
       <c r="D133" t="n">
-        <v>239.1088211458664</v>
+        <v>239.1088059824489</v>
       </c>
       <c r="E133" t="n">
-        <v>240.6127166748047</v>
+        <v>240.6127014160156</v>
       </c>
       <c r="F133" t="n">
         <v>7571500</v>
@@ -3930,16 +3930,16 @@
         <v>46099</v>
       </c>
       <c r="B135" t="n">
-        <v>235.349094010365</v>
+        <v>235.349078713635</v>
       </c>
       <c r="C135" t="n">
-        <v>236.5759581604242</v>
+        <v>236.5759427839531</v>
       </c>
       <c r="D135" t="n">
-        <v>232.9250616652477</v>
+        <v>232.9250465260699</v>
       </c>
       <c r="E135" t="n">
-        <v>234.7653503417969</v>
+        <v>234.7653350830078</v>
       </c>
       <c r="F135" t="n">
         <v>6811500</v>
@@ -4242,16 +4242,16 @@
         <v>46118</v>
       </c>
       <c r="B147" t="n">
-        <v>240.0784329225297</v>
+        <v>240.0784175573595</v>
       </c>
       <c r="C147" t="n">
-        <v>240.9392230850874</v>
+        <v>240.9392076648261</v>
       </c>
       <c r="D147" t="n">
-        <v>237.9512242744999</v>
+        <v>237.9512090454724</v>
       </c>
       <c r="E147" t="n">
-        <v>238.4162445068359</v>
+        <v>238.4162292480469</v>
       </c>
       <c r="F147" t="n">
         <v>4442400</v>
@@ -4450,16 +4450,16 @@
         <v>46128</v>
       </c>
       <c r="B155" t="n">
-        <v>234.9038500080299</v>
+        <v>234.9038654541874</v>
       </c>
       <c r="C155" t="n">
-        <v>235.6162207436799</v>
+        <v>235.6162362366795</v>
       </c>
       <c r="D155" t="n">
-        <v>229.6600157416919</v>
+        <v>229.6600308430398</v>
       </c>
       <c r="E155" t="n">
-        <v>232.0543670654297</v>
+        <v>232.0543823242188</v>
       </c>
       <c r="F155" t="n">
         <v>8668900</v>
@@ -4528,16 +4528,16 @@
         <v>46133</v>
       </c>
       <c r="B158" t="n">
-        <v>226.9193941968888</v>
+        <v>226.9193787228735</v>
       </c>
       <c r="C158" t="n">
-        <v>227.2557873120845</v>
+        <v>227.2557718151299</v>
       </c>
       <c r="D158" t="n">
-        <v>222.3186650386415</v>
+        <v>222.3186498783577</v>
       </c>
       <c r="E158" t="n">
-        <v>223.7631988525391</v>
+        <v>223.76318359375</v>
       </c>
       <c r="F158" t="n">
         <v>11681200</v>
@@ -4580,16 +4580,16 @@
         <v>46135</v>
       </c>
       <c r="B160" t="n">
-        <v>224.8416356959219</v>
+        <v>224.8416507297823</v>
       </c>
       <c r="C160" t="n">
-        <v>228.9377599403605</v>
+        <v>228.937775248105</v>
       </c>
       <c r="D160" t="n">
-        <v>224.6239660179549</v>
+        <v>224.623981037261</v>
       </c>
       <c r="E160" t="n">
-        <v>228.2055969238281</v>
+        <v>228.2056121826172</v>
       </c>
       <c r="F160" t="n">
         <v>7097600</v>
@@ -4606,16 +4606,16 @@
         <v>46136</v>
       </c>
       <c r="B161" t="n">
-        <v>226.6027887018479</v>
+        <v>226.6027733404394</v>
       </c>
       <c r="C161" t="n">
-        <v>227.5526214735122</v>
+        <v>227.5526060477145</v>
       </c>
       <c r="D161" t="n">
-        <v>224.6140956793093</v>
+        <v>224.6140804527143</v>
       </c>
       <c r="E161" t="n">
-        <v>225.0890045166016</v>
+        <v>225.0889892578125</v>
       </c>
       <c r="F161" t="n">
         <v>6067500</v>
@@ -4632,16 +4632,16 @@
         <v>46139</v>
       </c>
       <c r="B162" t="n">
-        <v>223.3773245484034</v>
+        <v>223.3773398363102</v>
       </c>
       <c r="C162" t="n">
-        <v>225.4946445162854</v>
+        <v>225.4946599491012</v>
       </c>
       <c r="D162" t="n">
-        <v>221.9723753264516</v>
+        <v>221.972390518204</v>
       </c>
       <c r="E162" t="n">
-        <v>222.9518737792969</v>
+        <v>222.9518890380859</v>
       </c>
       <c r="F162" t="n">
         <v>7897800</v>
@@ -4684,16 +4684,16 @@
         <v>46141</v>
       </c>
       <c r="B164" t="n">
-        <v>223.1299896858621</v>
+        <v>223.1299745498951</v>
       </c>
       <c r="C164" t="n">
-        <v>226.2861851379911</v>
+        <v>226.2861697879244</v>
       </c>
       <c r="D164" t="n">
-        <v>222.4769806067155</v>
+        <v>222.4769655150452</v>
       </c>
       <c r="E164" t="n">
-        <v>224.9405975341797</v>
+        <v>224.9405822753906</v>
       </c>
       <c r="F164" t="n">
         <v>7071100</v>
@@ -4840,16 +4840,16 @@
         <v>46149</v>
       </c>
       <c r="B170" t="n">
-        <v>222.3978024591847</v>
+        <v>222.397817873641</v>
       </c>
       <c r="C170" t="n">
-        <v>222.3978024591847</v>
+        <v>222.397817873641</v>
       </c>
       <c r="D170" t="n">
-        <v>218.2917897898664</v>
+        <v>218.2918049197337</v>
       </c>
       <c r="E170" t="n">
-        <v>220.15185546875</v>
+        <v>220.1518707275391</v>
       </c>
       <c r="F170" t="n">
         <v>7269700</v>
@@ -4918,16 +4918,16 @@
         <v>46154</v>
       </c>
       <c r="B173" t="n">
-        <v>220.6366899653626</v>
+        <v>220.6366747923043</v>
       </c>
       <c r="C173" t="n">
-        <v>225.2374041432973</v>
+        <v>225.2373886538506</v>
       </c>
       <c r="D173" t="n">
-        <v>219.3009909603728</v>
+        <v>219.3009758791698</v>
       </c>
       <c r="E173" t="n">
-        <v>221.8833312988281</v>
+        <v>221.8833160400391</v>
       </c>
       <c r="F173" t="n">
         <v>8632500</v>
@@ -4970,16 +4970,16 @@
         <v>46156</v>
       </c>
       <c r="B175" t="n">
-        <v>228.5518965755589</v>
+        <v>228.5519118475702</v>
       </c>
       <c r="C175" t="n">
-        <v>229.3038367743656</v>
+        <v>229.3038520966222</v>
       </c>
       <c r="D175" t="n">
-        <v>226.7314002434507</v>
+        <v>226.7314153938151</v>
       </c>
       <c r="E175" t="n">
-        <v>228.3540191650391</v>
+        <v>228.3540344238281</v>
       </c>
       <c r="F175" t="n">
         <v>6974400</v>
@@ -11102,7 +11102,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-07 03:08:29</t>
+          <t>2026-09-08 08:52:20</t>
         </is>
       </c>
     </row>

</xml_diff>